<commit_message>
Learnt New Dynamic Sliding Window Problems
</commit_message>
<xml_diff>
--- a/DSA Tracking Sheet.xlsx
+++ b/DSA Tracking Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Structures and Algorithm\Pattern_Based_DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D60F0D9-1B86-494A-BAE9-A7881FE620E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185BF15C-A265-4E82-96D3-ABD93FF48AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EA109011-75D6-4B4C-8940-30E2C0B9B007}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EA109011-75D6-4B4C-8940-30E2C0B9B007}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="111">
   <si>
     <t>Problem</t>
   </si>
@@ -345,6 +345,77 @@
 4. Problem involves comparing elements from both ends
 5. Two indices move through the array to reduce search space.
 6. In-place Modification is being asked</t>
+  </si>
+  <si>
+    <t>Trigger : Sorted array and comparison of positions</t>
+  </si>
+  <si>
+    <t>Result array is filled from the back because we are placing the largest square first
+i &lt; j is not the right loop condition here — use index &gt;= 0 to ensure all positions are filled</t>
+  </si>
+  <si>
+    <t>Array can be sorted and I could use Two Sum Approach</t>
+  </si>
+  <si>
+    <t>We just hold one element of array and apply Two Sum approach on it.</t>
+  </si>
+  <si>
+    <t>Make sure to handle the duplicates condition if asked in the question</t>
+  </si>
+  <si>
+    <t>O(n²)</t>
+  </si>
+  <si>
+    <t>Array | List&lt;List&gt;</t>
+  </si>
+  <si>
+    <t>Minimum Size Subarray Sum</t>
+  </si>
+  <si>
+    <t>Video</t>
+  </si>
+  <si>
+    <t>Subarray + minimum length -&gt; Dynamic Sliding Window</t>
+  </si>
+  <si>
+    <t>Dynamic Window</t>
+  </si>
+  <si>
+    <t>Even though there's a nested while loop, it's not O(n²) because low never resets — it only moves forward.</t>
+  </si>
+  <si>
+    <t>Use inner while loop not if — keep shrinking the window as long as sum &gt;= target to find minimum</t>
+  </si>
+  <si>
+    <t>Largest squares are always at either end. Use opposite end pointers, fill result array from right to left.
+In-place modification doesn't work because overwriting loses original values needed for comparison</t>
+  </si>
+  <si>
+    <t>Longest Substring with K Uniques</t>
+  </si>
+  <si>
+    <t>Longest Substring with At Least K Repeating Characters</t>
+  </si>
+  <si>
+    <t>Input is a string + find longest substring + constraint on K unique elements inside window → Dynamic Sliding Window</t>
+  </si>
+  <si>
+    <t>Array | Map</t>
+  </si>
+  <si>
+    <t>Shrink window from left when map.size() &gt; k — not when duplicates appear
+Decrement frequency first, then check if it became 0 before removing from map
+map.size() == k is the only valid state to update result</t>
+  </si>
+  <si>
+    <t>map.size() &lt; k → just expand, no action needed
+map.size() &gt; k → shrink from left until map size is back to k
+Return -1 as default result handles the case where no valid substring exists
+getOrDefault(ch, 0) + 1 — if character exists return its count, else return 0, then increment</t>
+  </si>
+  <si>
+    <t>O(k+1)
+since the map holds at most k+1 distinct characters at any point.</t>
   </si>
 </sst>
 </file>
@@ -405,7 +476,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -436,8 +507,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -452,19 +529,6 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -513,18 +577,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -536,6 +588,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -971,82 +1035,82 @@
   </cols>
   <sheetData>
     <row r="5" spans="2:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
     </row>
     <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="F6" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="H6" s="14" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="142.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="H7" s="19" t="s">
+      <c r="H7" s="15" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="171.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="20" t="s">
+      <c r="G8" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="H8" s="19" t="s">
+      <c r="H8" s="15" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1066,11 +1130,13 @@
     <col min="1" max="1" width="31.21875" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.33203125" customWidth="1"/>
-    <col min="4" max="4" width="21.109375" customWidth="1"/>
-    <col min="5" max="5" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.88671875" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" customWidth="1"/>
     <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.21875" customWidth="1"/>
-    <col min="8" max="11" width="25.88671875" customWidth="1"/>
+    <col min="8" max="9" width="25.88671875" customWidth="1"/>
+    <col min="10" max="10" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12" customWidth="1"/>
     <col min="13" max="13" width="15.33203125" customWidth="1"/>
     <col min="14" max="14" width="15.44140625" customWidth="1"/>
@@ -1218,55 +1284,91 @@
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
+      <c r="C4" s="2">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>82</v>
+      </c>
       <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M4" s="1"/>
+      <c r="F4" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K4" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M4" s="18">
+        <v>46089</v>
+      </c>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
+        <v>63</v>
+      </c>
+      <c r="C5" s="2">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="E5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M5" s="1"/>
+        <v>96</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M5" s="18">
+        <v>46091</v>
+      </c>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
@@ -1657,15 +1759,15 @@
   <dimension ref="A1:Q22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.33203125" customWidth="1"/>
     <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.44140625" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="36.44140625" customWidth="1"/>
     <col min="7" max="7" width="15" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.21875" customWidth="1"/>
-    <col min="9" max="9" width="23" customWidth="1"/>
+    <col min="8" max="8" width="39.44140625" customWidth="1"/>
+    <col min="9" max="9" width="31.6640625" customWidth="1"/>
     <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="6.21875" bestFit="1" customWidth="1"/>
@@ -1725,7 +1827,7 @@
       </c>
     </row>
     <row r="2" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="10" t="s">
         <v>33</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1768,7 +1870,7 @@
       <c r="Q2" s="7"/>
     </row>
     <row r="3" spans="1:17" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="20" t="s">
         <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1783,7 +1885,7 @@
       <c r="E3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="13" t="s">
         <v>73</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -1811,7 +1913,7 @@
       <c r="Q3" s="9"/>
     </row>
     <row r="4" spans="1:17" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="20" t="s">
         <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1826,7 +1928,7 @@
       <c r="E4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="13" t="s">
         <v>73</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -1853,56 +1955,108 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="1"/>
+    <row r="5" spans="1:17" ht="72" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="2">
+        <v>30</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K5" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4"/>
-      <c r="K6" s="4"/>
-      <c r="L6" s="1"/>
+    <row r="6" spans="1:17" ht="144" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="2">
+        <v>40</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="I6" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4"/>
-      <c r="K7" s="4"/>
+    <row r="7" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -1911,17 +2065,17 @@
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
+      <c r="A8" s="20"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
@@ -1930,17 +2084,17 @@
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="A9" s="20"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
@@ -1949,17 +2103,17 @@
       <c r="Q9" s="1"/>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4"/>
-      <c r="K10" s="4"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
@@ -1968,17 +2122,17 @@
       <c r="Q10" s="1"/>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4"/>
-      <c r="K11" s="4"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
@@ -1987,17 +2141,17 @@
       <c r="Q11" s="1"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
+      <c r="A12" s="20"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="1"/>
@@ -2006,17 +2160,17 @@
       <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
+      <c r="A13" s="20"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
@@ -2026,16 +2180,16 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="10"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="1"/>
@@ -2044,17 +2198,17 @@
       <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
+      <c r="A15" s="20"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
@@ -2063,17 +2217,17 @@
       <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
+      <c r="A16" s="20"/>
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
@@ -2083,16 +2237,16 @@
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
@@ -2101,12 +2255,12 @@
       <c r="Q17" s="1"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
+      <c r="A18" s="20"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -2120,12 +2274,12 @@
       <c r="Q18" s="1"/>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="A19" s="20"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -2139,12 +2293,12 @@
       <c r="Q19" s="1"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
+      <c r="A20" s="20"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -2158,12 +2312,12 @@
       <c r="Q20" s="1"/>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
+      <c r="A21" s="20"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -2177,12 +2331,12 @@
       <c r="Q21" s="1"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="A22" s="20"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
@@ -2200,8 +2354,11 @@
     <hyperlink ref="A2" r:id="rId1" xr:uid="{F0E6F405-EB37-4CA7-A358-5C666F410C53}"/>
     <hyperlink ref="A3" r:id="rId2" xr:uid="{2BCB52B1-9CB6-494C-9F8E-890F1DD4D441}"/>
     <hyperlink ref="A4" r:id="rId3" display="https://leetcode.com/problems/maximum-sum-of-distinct-subarrays-with-length-k/" xr:uid="{4CDD9DB7-8216-4628-895A-252CDC46323E}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://leetcode.com/problems/minimum-size-subarray-sum/" xr:uid="{87D89978-DEC6-4FE3-9F53-3AFE52A15A93}"/>
+    <hyperlink ref="A6" r:id="rId5" xr:uid="{4DBED0AB-BA0A-4904-AE72-1D2F538572E8}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://leetcode.com/problems/longest-substring-with-at-least-k-repeating-characters/" xr:uid="{5A07E760-C3F5-431C-ADA6-C6958C0C4F79}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Solved Hard Sliding Window Problems
</commit_message>
<xml_diff>
--- a/DSA Tracking Sheet.xlsx
+++ b/DSA Tracking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Structures and Algorithm\Pattern_Based_DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185BF15C-A265-4E82-96D3-ABD93FF48AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68DAC298-4FC1-4973-91BE-EF2A8206A856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{EA109011-75D6-4B4C-8940-30E2C0B9B007}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="130">
   <si>
     <t>Problem</t>
   </si>
@@ -416,6 +416,78 @@
   <si>
     <t>O(k+1)
 since the map holds at most k+1 distinct characters at any point.</t>
+  </si>
+  <si>
+    <t>Fruit Into Baskets</t>
+  </si>
+  <si>
+    <t>O(1)
+The map holds at most 3 entries at any point — you remove when size exceeds 2. So space is O(1) (or O(k) where k=2, which is constant)</t>
+  </si>
+  <si>
+    <t>Two baskets = at most 2 distinct values → Dynamic Sliding Window + HashMap
+This is identical to Longest K Distinct Characters with k=2
+Shrink window from left when map.size() &gt; 2, update result when map.size() &lt;= 2</t>
+  </si>
+  <si>
+    <t>Initialize maxLength with Integer.MIN_VALUE — but be careful, if all windows have less than 2 distinct types, == 2 condition never triggers. Use &lt;= 2 to handle arrays with only 1 distinct fruit type</t>
+  </si>
+  <si>
+    <t>input is an array + find the longest subarray with at most 2 distinct number</t>
+  </si>
+  <si>
+    <t>Longest Substring Without Repeating Characters</t>
+  </si>
+  <si>
+    <t>input is an array + find the longest subarray with unique characters</t>
+  </si>
+  <si>
+    <t>Window becomes invalid when any character's frequency &gt; 1, not when map.size() exceeds something
+Use while not if for shrinking — if only removes one character from left, but the duplicate may not be at low
+Update maxLen after every shrink — at that point window is guaranteed valid</t>
+  </si>
+  <si>
+    <t>Space is O(1) not O(n) — map is bounded by character set size (26 for lowercase, 128 for ASCII)
+Key difference from previous problems: invalid condition is frequency based, not map size based
+Shrink continues until the duplicate character is actually removed from the window</t>
+  </si>
+  <si>
+    <t>Longest Repeating Character Replacement</t>
+  </si>
+  <si>
+    <t>Hard</t>
+  </si>
+  <si>
+    <t>input is string + find the longest substring with a condition</t>
+  </si>
+  <si>
+    <t>Space is O(1) — map bounded by 26 uppercase characters, not input size
+Use while not if for shrinking — window may need multiple shrinks before becoming valid
+You don't actually perform replacements — you just check if it's feasible within k operations</t>
+  </si>
+  <si>
+    <t>Minimum Window Substring</t>
+  </si>
+  <si>
+    <t>AI + Video</t>
+  </si>
+  <si>
+    <t>input is string + find the shortest substring with a condition</t>
+  </si>
+  <si>
+    <t>Use required counter starting at t.length() — decrements when windowFreq &lt;= tFreq for a needed char, increments when shrinking drops a char below required frequency
+Window is valid when required == 0
+Record window only when current length &lt; minLen — not on every valid window
+Use s.substring(low, high + 1) not s.substring(low, low + minLen) — minLen may be from a previous smaller window</t>
+  </si>
+  <si>
+    <t>windowFreq &lt;= tFreq condition handles duplicates — for t = "aaa", required decrements 3 times as a frequency grows from 1 to 3
+During shrink, required++ only when tMap.containsKey(char) AND windowFreq drops below tFreq — not just when frequency hits 0
+This is harder than it looks — the required counter is the key insight that avoids comparing two full maps at every step
+Space O(1) — both maps bounded by 52 characters (26 uppercase + 26 lowercase)</t>
+  </si>
+  <si>
+    <t>O(m+n)</t>
   </si>
 </sst>
 </file>
@@ -542,7 +614,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -592,14 +664,23 @@
     <xf numFmtId="15" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1035,15 +1116,15 @@
   </cols>
   <sheetData>
     <row r="5" spans="2:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="23"/>
     </row>
     <row r="6" spans="2:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="14" t="s">
@@ -1869,8 +1950,8 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
+    <row r="3" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1912,8 +1993,8 @@
       <c r="P3" s="9"/>
       <c r="Q3" s="9"/>
     </row>
-    <row r="4" spans="1:17" ht="72" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+    <row r="4" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
         <v>35</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1955,8 +2036,8 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:17" ht="72" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
         <v>97</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1999,7 +2080,7 @@
       <c r="Q5" s="1"/>
     </row>
     <row r="6" spans="1:17" ht="144" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>104</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -2042,7 +2123,7 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="20" t="s">
         <v>105</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -2055,8 +2136,6 @@
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
@@ -2064,76 +2143,172 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A8" s="20"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
+    <row r="8" spans="1:17" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="2">
+        <v>15</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K8" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M8" s="1"/>
       <c r="N8" s="1"/>
       <c r="O8" s="1"/>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A9" s="20"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
+    <row r="9" spans="1:17" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="2">
+        <v>30</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M9" s="1"/>
       <c r="N9" s="1"/>
       <c r="O9" s="1"/>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="20"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
+    <row r="10" spans="1:17" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C10" s="2">
+        <v>50</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L10" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M10" s="1"/>
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A11" s="20"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
+    <row r="11" spans="1:17" ht="216" x14ac:dyDescent="0.3">
+      <c r="A11" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C11" s="2">
+        <v>70</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="G11" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L11" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="M11" s="1"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
@@ -2141,7 +2316,7 @@
       <c r="Q11" s="1"/>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A12" s="20"/>
+      <c r="A12" s="19"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -2160,7 +2335,7 @@
       <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A13" s="20"/>
+      <c r="A13" s="19"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -2198,7 +2373,7 @@
       <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A15" s="20"/>
+      <c r="A15" s="19"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -2217,7 +2392,7 @@
       <c r="Q15" s="1"/>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A16" s="20"/>
+      <c r="A16" s="19"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -2255,7 +2430,7 @@
       <c r="Q17" s="1"/>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A18" s="20"/>
+      <c r="A18" s="19"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -2274,7 +2449,7 @@
       <c r="Q18" s="1"/>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A19" s="20"/>
+      <c r="A19" s="19"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -2293,7 +2468,7 @@
       <c r="Q19" s="1"/>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A20" s="20"/>
+      <c r="A20" s="19"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -2312,7 +2487,7 @@
       <c r="Q20" s="1"/>
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A21" s="20"/>
+      <c r="A21" s="19"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -2331,7 +2506,7 @@
       <c r="Q21" s="1"/>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A22" s="20"/>
+      <c r="A22" s="19"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -2357,8 +2532,12 @@
     <hyperlink ref="A5" r:id="rId4" display="https://leetcode.com/problems/minimum-size-subarray-sum/" xr:uid="{87D89978-DEC6-4FE3-9F53-3AFE52A15A93}"/>
     <hyperlink ref="A6" r:id="rId5" xr:uid="{4DBED0AB-BA0A-4904-AE72-1D2F538572E8}"/>
     <hyperlink ref="A7" r:id="rId6" display="https://leetcode.com/problems/longest-substring-with-at-least-k-repeating-characters/" xr:uid="{5A07E760-C3F5-431C-ADA6-C6958C0C4F79}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://leetcode.com/problems/fruit-into-baskets/" xr:uid="{F73B731F-FF91-4C17-A873-E2F13B1BF745}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://leetcode.com/problems/longest-substring-without-repeating-characters/" xr:uid="{77937BF3-2DD6-4846-8E8D-B36466EE3597}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://leetcode.com/problems/longest-repeating-character-replacement/" xr:uid="{0D5423E5-349D-410E-BA09-77EF8855B792}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://leetcode.com/problems/minimum-window-substring/" xr:uid="{2CFF3C27-EA43-4238-8246-53038B73E0F3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId7"/>
+  <drawing r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>